<commit_message>
vlookup and hlookup index and match
</commit_message>
<xml_diff>
--- a/t388_excel.xlsx
+++ b/t388_excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinay chidapareddi\OneDrive\Documents\T388_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB9116D-4F10-4BC6-931B-9B1F4C94C96F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2B25267-78D7-4D04-BD02-F23AF6E0B4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A8B67965-C95B-4B3E-A167-91AF85600403}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{A8B67965-C95B-4B3E-A167-91AF85600403}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
@@ -36,8 +36,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="66">
   <si>
     <t>name</t>
   </si>
@@ -229,13 +251,19 @@
   </si>
   <si>
     <t>vegetable</t>
+  </si>
+  <si>
+    <t>remark</t>
+  </si>
+  <si>
+    <t>Grade</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -262,6 +290,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -316,11 +351,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -333,21 +369,27 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
@@ -2013,18 +2055,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E66F7C91-6B57-44BC-9223-39A3F1B9349F}">
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="37.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.90625" customWidth="1"/>
+    <col min="10" max="10" width="37.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
@@ -2046,11 +2089,17 @@
       <c r="G1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="H1" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="K1" s="6" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L1" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2074,17 +2123,25 @@
       <c r="G2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="12" t="str">
+        <f>IF(F2&gt;=47000,"extraordinary","average")</f>
+        <v>average</v>
+      </c>
+      <c r="I2" t="s">
         <v>13</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L2" t="str">
+        <f>IF(F2&gt;=55000,"Excellent salary",IF(F2&gt;=50000,"regular salary",IF(F2&gt;45000,"Normal salary","less salary")))</f>
+        <v>less salary</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -2108,17 +2165,25 @@
       <c r="G3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="12" t="str">
+        <f t="shared" ref="H3:H7" si="2">IF(F3&gt;=47000,"extraordinary","average")</f>
+        <v>extraordinary</v>
+      </c>
+      <c r="I3" t="s">
         <v>7</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L3" t="str">
+        <f t="shared" ref="L3:L7" si="3">IF(F3&gt;=55000,"Excellent salary",IF(F3&gt;=50000,"regular salary",IF(F3&gt;45000,"Normal salary","less salary")))</f>
+        <v>Normal salary</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -2142,17 +2207,25 @@
       <c r="G4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>average</v>
+      </c>
+      <c r="I4" t="s">
         <v>11</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L4" t="str">
+        <f t="shared" si="3"/>
+        <v>less salary</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -2176,17 +2249,25 @@
       <c r="G5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>extraordinary</v>
+      </c>
+      <c r="I5" t="s">
         <v>15</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L5" t="str">
+        <f t="shared" si="3"/>
+        <v>regular salary</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -2210,17 +2291,25 @@
       <c r="G6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>average</v>
+      </c>
+      <c r="I6" t="s">
         <v>21</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="K6" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="L6" t="str">
+        <f t="shared" si="3"/>
+        <v>less salary</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -2244,25 +2333,33 @@
       <c r="G7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>extraordinary</v>
+      </c>
+      <c r="I7" t="s">
         <v>23</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>24</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="K7" s="4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="H8" t="s">
+      <c r="L7" t="str">
+        <f t="shared" si="3"/>
+        <v>Excellent salary</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="I8" t="s">
         <v>37</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
@@ -2272,8 +2369,11 @@
       <c r="C9" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>1</v>
       </c>
@@ -2283,8 +2383,12 @@
       <c r="C10" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D10" s="13">
+        <f>C10/$F$9</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>2</v>
       </c>
@@ -2294,8 +2398,12 @@
       <c r="C11" s="7">
         <v>15</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D11" s="13">
+        <f t="shared" ref="D11:D19" si="4">C11/$F$9</f>
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>3</v>
       </c>
@@ -2305,8 +2413,16 @@
       <c r="C12" s="7">
         <v>35</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D12" s="13">
+        <f t="shared" si="4"/>
+        <v>0.35</v>
+      </c>
+      <c r="E12" t="e" cm="1">
+        <f t="array" ref="E12">SU</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>4</v>
       </c>
@@ -2316,8 +2432,19 @@
       <c r="C13" s="7">
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D13" s="13">
+        <f t="shared" si="4"/>
+        <v>0.2</v>
+      </c>
+      <c r="E13">
+        <v>51</v>
+      </c>
+      <c r="F13" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(H2)</f>
+        <v>=IF(F2&gt;=47000,"extraordinary","average")</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>5</v>
       </c>
@@ -2327,8 +2454,19 @@
       <c r="C14" s="7">
         <v>30</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D14" s="13">
+        <f t="shared" si="4"/>
+        <v>0.3</v>
+      </c>
+      <c r="E14">
+        <v>52</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" ref="F14:F19" ca="1" si="5">_xlfn.FORMULATEXT(H3)</f>
+        <v>=IF(F3&gt;=47000,"extraordinary","average")</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>6</v>
       </c>
@@ -2338,8 +2476,19 @@
       <c r="C15" s="7">
         <v>40</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="D15" s="13">
+        <f t="shared" si="4"/>
+        <v>0.4</v>
+      </c>
+      <c r="E15">
+        <v>53</v>
+      </c>
+      <c r="F15" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v>=IF(F4&gt;=47000,"extraordinary","average")</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>1</v>
       </c>
@@ -2349,8 +2498,19 @@
       <c r="C16" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D16" s="13">
+        <f t="shared" si="4"/>
+        <v>0.1</v>
+      </c>
+      <c r="E16">
+        <v>54</v>
+      </c>
+      <c r="F16" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v>=IF(F5&gt;=47000,"extraordinary","average")</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>2</v>
       </c>
@@ -2360,8 +2520,19 @@
       <c r="C17" s="7">
         <v>65</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D17" s="13">
+        <f t="shared" si="4"/>
+        <v>0.65</v>
+      </c>
+      <c r="E17">
+        <v>51</v>
+      </c>
+      <c r="F17" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v>=IF(F6&gt;=47000,"extraordinary","average")</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>1</v>
       </c>
@@ -2371,8 +2542,19 @@
       <c r="C18" s="7">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D18" s="13">
+        <f t="shared" si="4"/>
+        <v>0.1</v>
+      </c>
+      <c r="E18">
+        <v>52</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v>=IF(F7&gt;=47000,"extraordinary","average")</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>5</v>
       </c>
@@ -2382,8 +2564,19 @@
       <c r="C19" s="7">
         <v>50</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D19" s="13">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="E19">
+        <v>59</v>
+      </c>
+      <c r="F19" t="e">
+        <f t="shared" ca="1" si="5"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -2391,7 +2584,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="9">
         <v>46023</v>
       </c>
@@ -2399,7 +2592,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="9">
         <v>46054</v>
       </c>
@@ -2407,7 +2600,7 @@
         <v>206.7</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="9">
         <v>46082</v>
       </c>
@@ -2415,7 +2608,7 @@
         <v>204.3</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="9">
         <v>46113</v>
       </c>
@@ -2423,7 +2616,7 @@
         <v>207.8</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="9">
         <v>46143</v>
       </c>
@@ -2431,7 +2624,7 @@
         <v>208.1</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="9">
         <v>46174</v>
       </c>
@@ -2439,7 +2632,7 @@
         <v>207.9</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="9">
         <v>46204</v>
       </c>
@@ -2447,19 +2640,19 @@
         <v>208.2</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="9">
         <v>46235</v>
       </c>
     </row>
-    <row r="37" spans="6:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="6:9" x14ac:dyDescent="0.35">
       <c r="F37">
         <v>10</v>
       </c>
       <c r="G37">
         <v>5</v>
       </c>
-      <c r="H37">
+      <c r="I37">
         <f>F37*G37</f>
         <v>50</v>
       </c>
@@ -2473,12 +2666,12 @@
     <hyperlink ref="G5" r:id="rId4" xr:uid="{77CE4FCA-2919-4415-9C17-694768B2EBF0}"/>
     <hyperlink ref="G6" r:id="rId5" xr:uid="{7F7B7DED-F3FB-437A-BA87-7EC418148225}"/>
     <hyperlink ref="G7" r:id="rId6" xr:uid="{C4985332-BA31-4F46-B2BC-E758F7EDEF22}"/>
-    <hyperlink ref="J2" r:id="rId7" xr:uid="{FE092D4F-65DC-4F04-A21A-C17CB1E10C40}"/>
-    <hyperlink ref="J3" r:id="rId8" xr:uid="{1CEE6724-62D8-401B-88A2-C22863B4DD7C}"/>
-    <hyperlink ref="J4" r:id="rId9" xr:uid="{706E93D7-1828-44A4-823B-7817A9A53D1B}"/>
-    <hyperlink ref="J5" r:id="rId10" xr:uid="{AF606569-9795-45E2-92D5-74E21A633DF7}"/>
-    <hyperlink ref="J6" r:id="rId11" xr:uid="{909BADDA-4B17-45DB-9905-51665FA9A6B8}"/>
-    <hyperlink ref="J7" r:id="rId12" xr:uid="{2DDDA12C-E26E-4482-9FFF-46BD2A62A26E}"/>
+    <hyperlink ref="K2" r:id="rId7" xr:uid="{FE092D4F-65DC-4F04-A21A-C17CB1E10C40}"/>
+    <hyperlink ref="K3" r:id="rId8" xr:uid="{1CEE6724-62D8-401B-88A2-C22863B4DD7C}"/>
+    <hyperlink ref="K4" r:id="rId9" xr:uid="{706E93D7-1828-44A4-823B-7817A9A53D1B}"/>
+    <hyperlink ref="K5" r:id="rId10" xr:uid="{AF606569-9795-45E2-92D5-74E21A633DF7}"/>
+    <hyperlink ref="K6" r:id="rId11" xr:uid="{909BADDA-4B17-45DB-9905-51665FA9A6B8}"/>
+    <hyperlink ref="K7" r:id="rId12" xr:uid="{2DDDA12C-E26E-4482-9FFF-46BD2A62A26E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>